<commit_message>
update translated notion exports 2026-06-26T14:03:17
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,50 +454,60 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>abstract_zh</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>topics</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>keywords</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>reading_status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>processing_status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>translation_status</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>priority</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>use_type</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>related_chapter</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>notion_page_id</t>
         </is>

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T14:36:09
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y3"/>
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,248 +424,127 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>export_enabled</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>title_zh</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>authors</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>doi</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>abstract</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>abstract_zh</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>topics</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>keywords</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>use_type</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>related_chapter</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>priority</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>reading_status</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>translation_status</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>derived_translation_status</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>processing_status</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>derived_processing_status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>claim_supported</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>notion_writeback_status</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>material_pack_status</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>notion_page_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-06-26T14:32:16</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Untitled</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>待翻译</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>待翻译</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>待补充信息</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>待补充信息</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>skipped_existing_or_no_fields</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>https://app.notion.com/p/38be8c8a654d801fad96c5603f7f69f5</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>38be8c8a-654d-801f-ad96-c5603f7f69f5</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-06-26T14:32:16</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Untitled</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>待翻译</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>待翻译</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>待补充信息</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>待补充信息</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>skipped_existing_or_no_fields</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>https://app.notion.com/p/38be8c8a654d80c1a227fbff84e12200</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>38be8c8a-654d-80c1-a227-fbff84e12200</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T17:58:40
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -551,7 +551,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T17:53:16</t>
+          <t>2026-06-26T17:58:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T17:53:16</t>
+          <t>2026-06-26T17:58:40</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -743,7 +743,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T17:53:16</t>
+          <t>2026-06-26T17:58:40</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -839,7 +839,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T17:53:16</t>
+          <t>2026-06-26T17:58:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -931,7 +931,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T17:53:16</t>
+          <t>2026-06-26T17:58:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1023,7 +1023,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T17:53:16</t>
+          <t>2026-06-26T17:58:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T18:33:25
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -596,7 +596,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T18:24:06</t>
+          <t>2026-06-26T18:33:25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -715,7 +715,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T18:24:06</t>
+          <t>2026-06-26T18:33:25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -834,7 +834,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T18:24:06</t>
+          <t>2026-06-26T18:33:25</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -953,7 +953,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T18:24:06</t>
+          <t>2026-06-26T18:33:25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1068,7 +1068,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T18:24:06</t>
+          <t>2026-06-26T18:33:25</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T18:24:06</t>
+          <t>2026-06-26T18:33:25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-06-26T18:58:21
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -596,7 +596,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-26T18:50:39</t>
+          <t>2026-06-26T18:58:21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -609,7 +609,11 @@
           <t>The link between perceived human resource management practices, engagement and employee behaviour: a moderated mediation model</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>感知人力资源管理实践、敬业度与员工行为之间的联系：一个有调节的中介模型</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>K. Alfes; A. D. Shantz; C. Truss; E. C. Soane</t>
@@ -635,7 +639,11 @@
           <t>This study contributes to our understanding of the mediating and moderating processes through which human resource management practices are linked with behavioural outcomes. We developed and tested a moderated mediation model linking perceived human resource management practices to organisational citizenship behaviour and turnover intentions. Drawing on social exchange theory, our model posits that the effect of perceived human resource management practices on both outcome variables is mediated by levels of employee engagement, while the relationship between employee engagement and both outcome variables is moderated by perceived organisational support and leader-member exchange. Overall, data from 297 employees in a service sector organisation in the UK support this model. This suggests that the enactment of positive behavioural outcomes, as a consequence of engagement, largely depends on the wider organisational climate and employees’ relationship with their line manager. Implications for practice and directions for future research are discussed.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>本研究有助于深化我们对人力资源管理实践与行为结果之间中介和调节过程的理解。我们构建并检验了一个调节中介模型，将感知到的人力资源管理实践与组织公民行为和离职意向联系起来。基于社会交换理论，本模型认为，感知到的人力资源管理实践对这两个结果变量的影响由员工敬业度水平所中介，而员工敬业度与这两个结果变量之间的关系受到感知到的组织支持和领导—成员交换的调节。总体而言，来自英国一家服务业组织297名员工的数据支持了该模型。这表明，作为敬业度结果的积极行为结果的实施，在很大程度上取决于更广泛的组织氛围以及员工与其直线经理的关系。文中讨论了对实践的启示以及未来研究方向。</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>to-notion</t>
@@ -648,12 +656,12 @@
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>已翻译</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>已翻译</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -663,7 +671,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>已同步</t>
+          <t>已导出</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -715,7 +723,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-26T18:50:39</t>
+          <t>2026-06-26T18:58:21</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -728,7 +736,11 @@
           <t>Allocative efficiency in public research funding: Can bibliometrics help?</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>公共研究资助中的配置效率：文献计量学能否提供帮助？</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>Giovanni Abramo; Ciriaco Andrea D’Angelo; Alessandro Caprasecca</t>
@@ -754,7 +766,11 @@
           <t>The use of outcome control modes of research evaluation exercises is ever more frequent. They are conceived as tools to stimulate increased levels of research productivity, and to guide choices in allocating components of government research budgets for publicly funded institutions. There are several contributions in the literature that compare the different methodological approaches that policy makers could adopt for these exercises, however the comparisons are limited to only a few disciplines. This work, examining the case of the whole of the “hard sciences” of the Italian academic system, makes a comparison between results obtained from peer review type of evaluations (as adopted by the Ministry of Universities and Research) and those possible from a bibliometric approach (as developed by the authors). The aim is to understand to what extent bibliometric methodology, which is noted as relatively inexpensive, time-saving and exhaustive, can complement and integrate peer review methodology in research evaluation.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>研究评价活动中成果控制模式的使用日益频繁。它们被构想为旨在促进研究生产力水平提高，并指导公共资助机构政府研究预算组成部分配置选择的工具。文献中已有若干研究比较了政策制定者可在此类评价活动中采用的不同方法路径，然而这些比较仅限于少数学科。本文考察意大利学术体系中整个“硬科学”领域的案例，比较了同行评议式评价（如大学与研究部所采用）所得结果与文献计量方法（由作者开发）可能获得的结果。其目的在于理解文献计量方法在多大程度上能够补充并整合同行评议方法用于研究评价；该方法被认为相对低成本、省时且覆盖全面。</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>to-notion</t>
@@ -767,12 +783,12 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>已翻译</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>已翻译</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -782,7 +798,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>已同步</t>
+          <t>已导出</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
@@ -834,7 +850,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-26T18:50:39</t>
+          <t>2026-06-26T18:58:21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -847,7 +863,11 @@
           <t>Consumer attitudes toward marketplace globalization: Structure, antecedents and consequences</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>消费者对市场全球化的态度：结构、前因与后果</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Dana L. Alden; Jan-Benedict E.M. Steenkamp; Rajeev Batra</t>
@@ -873,7 +893,11 @@
           <t>This study examines relationships between a new measure of consumer attitudes toward consumption alternatives resulting from market globalization, several attitudinal antecedents (materialism, susceptibility to normative influence and consumer ethnocentrism), and a hypothesized consequence of these attitudes — preference for global brands. Following validation of the new measure in three culturally distinct markets, South Korea, the US, and China, the hypothesized antecedents and consequence are tested in South Korea. Empirical findings broadly support hypotheses and provide important implications for future research on market globalization.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>本研究考察了一项衡量消费者对市场全球化所带来的消费替代选择之态度的新指标，与若干态度前因（物质主义、规范性影响易感性和消费者民族中心主义）以及这些态度的一个假设后果——对全球品牌的偏好——之间的关系。在韩国、美国和中国三个文化差异显著的市场中对该新指标进行验证后，研究在韩国检验了所假设的前因与后果。实证结果总体支持研究假设，并为未来关于市场全球化的研究提供了重要启示。</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>to-notion</t>
@@ -886,12 +910,12 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>已翻译</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>已翻译</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -901,7 +925,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>已同步</t>
+          <t>已导出</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
@@ -953,7 +977,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-26T18:50:39</t>
+          <t>2026-06-26T18:58:21</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -966,7 +990,11 @@
           <t>The Brand Relationship Spectrum: The Key to the Brand Architecture Challenge</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>品牌关系谱系：品牌架构挑战的关键</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>David A. Aaker; Erich Joachimsthaler</t>
@@ -1009,12 +1037,12 @@
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>已翻译</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>部分已翻译</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -1076,7 +1104,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-26T18:50:39</t>
+          <t>2026-06-26T18:58:21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1089,7 +1117,11 @@
           <t>Measuring Brand Equity Across Products and Markets</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>跨产品与市场的品牌资产测量</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>David A. Aaker</t>
@@ -1132,12 +1164,12 @@
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>已翻译</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>部分已翻译</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1199,7 +1231,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-26T18:50:39</t>
+          <t>2026-06-26T18:58:21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1212,7 +1244,11 @@
           <t>Leveraging the Corporate Brand</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>利用企业品牌</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>David A Aaker</t>
@@ -1243,12 +1279,12 @@
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>已翻译</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>待翻译</t>
+          <t>部分已翻译</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-07-07T09:23:33
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI1"/>
+  <dimension ref="A1:AI4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,6 +590,376 @@
       <c r="AI1" t="inlineStr">
         <is>
           <t>notion_page_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-07T09:23:33</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Trends in Theory Building and Theory Testing: A Five-Decade Study of the &lt;i&gt;Academy of Management Journal&lt;/i&gt;</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>理论建构与理论检验的趋势：基于《管理学会期刊》五十年的研究</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Jason A. Colquitt; Cindy P. Zapata-Phelan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Academy of Management Journal</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>10.5465/amj.2007.28165855</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>to-notion</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>已翻译</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>部分已翻译</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>已从 Zotero 导入</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>已同步</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="n">
+        <v>69</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>0. 文献名称
+TRENDS IN THEORY BUILDING AND THEORY TESTING: A  FIVE-DECADE STUDY OF THE ACADEMY OF  MANAGEMENT JOURNAL
+1. 研究并解决的问题
+研究问题：我们从理论构建和理论检验两个维度介绍一个反映实证文献理论贡献的分类法。
+现实痛点/理论缺口：尽管有多种因素可以解释这一趋势，但一个可能的原因是实证文章缺乏充分描述一个理论(大麦, 2006)要素所需的空间。考虑到这一局限性，一篇实证文章究竟意味着什么，才能做出理论上的贡献。
+作者要“解决”的具体点：我们的研究目的有三。首先，我们创建了一个</t>
+        </is>
+      </c>
+      <c r="AA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>skipped_existing_or_no_fields</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/Trends-in-Theory-Building-and-Theory-Testing-A-Five-Decade-Study-of-the-i-Academy-of-Management-Jo-395e8c8a654d815583dedaab8009b7b9</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>395e8c8a-654d-8155-83de-daab8009b7b9</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-07T09:23:33</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Methodological fit in management field research</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>管理领域研究中的方法论契合度</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Amy C. Edmondson; Stacy E. Mcmanus</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Academy of Management Review</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>10.5465/amr.2007.26586086</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>to-notion</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>已翻译</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>部分已翻译</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>已从 Zotero 导入</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>已同步</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="n">
+        <v>69</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>0. 文献名称
+Methodological fit in management field research
+1. 研究问题（Research Question）
+核心研究问题：方法匹配作为组织高质量实地研究的隐性价值属性，在管理学文献中很少受到关注。引入了一个权变框架，将先前的工作与研究项目的设计联系起来，特别关注在一篇研究论文中何时混合定性和定量数据的问题
+研究动机/现实背景：
+为了推进管理理论的发展，越来越多的学者从事实地研究，研究现实的人、现实的问题、现实的组织。虽然实地研究的潜在相关性是令人鼓舞的，但研究旅程可能是混乱和低效的，充满了逻辑障碍和意想不到的事件。研究人员管理与网站的复</t>
+        </is>
+      </c>
+      <c r="AA3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>skipped_existing_or_no_fields</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/Methodological-fit-in-management-field-research-395e8c8a654d81b69d3cce24cb21dc3a</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>395e8c8a-654d-81b6-9d3c-ce24cb21dc3a</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-07T09:23:33</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Building Theories from Case Study Research</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>从案例研究中构建理论</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kathleen M Eisenhardt</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>to-notion</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>已翻译</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>部分已翻译</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>已从 Zotero 导入</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>已同步</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="n">
+        <v>132</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>0. 文献名称
+Building Theories from Case  Study Research
+1. 研究并解决的问题
+研究问题：本文描述了运用案例研究进行理论归纳的过程- -从明确研究问题到得出研究结论。该过程的一些特征，如问题界定、构念验证等，与假设检验研究有相似之处。另外一些，如案例内分析和复制逻辑，是归纳的、面向案例的过程所特有的。总的来说，这里描述的过程是高度迭代的，并且与数据紧密相连。这种研究方法在新的主题领域尤其适用。由此产生的理论往往是新颖的、可检验的和经验有效的。最后，卢德分子的洞见、(例如,简约性、逻辑连贯性)的良好理论的检验以及证据中的令人信服的基础是评价这类研究</t>
+        </is>
+      </c>
+      <c r="AA4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>skipped_existing_or_no_fields</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>https://app.notion.com/p/Building-Theories-from-Case-Study-Research-395e8c8a654d814f96e6f7022871fd51</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>395e8c8a-654d-814f-96e6-f7022871fd51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update filtered material packs and word drafts 2026-07-07T14:57:45
</commit_message>
<xml_diff>
--- a/exports/literature_notes.xlsx
+++ b/exports/literature_notes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI4"/>
+  <dimension ref="A1:AI1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,376 +590,6 @@
       <c r="AI1" t="inlineStr">
         <is>
           <t>notion_page_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:23:33</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Trends in Theory Building and Theory Testing: A Five-Decade Study of the &lt;i&gt;Academy of Management Journal&lt;/i&gt;</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>理论建构与理论检验的趋势：基于《管理学会期刊》五十年的研究</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Jason A. Colquitt; Cindy P. Zapata-Phelan</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2007</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Academy of Management Journal</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>10.5465/amj.2007.28165855</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>to-notion</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>已翻译</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>部分已翻译</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>已从 Zotero 导入</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>已同步</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="n">
-        <v>69</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>0. 文献名称
-TRENDS IN THEORY BUILDING AND THEORY TESTING: A  FIVE-DECADE STUDY OF THE ACADEMY OF  MANAGEMENT JOURNAL
-1. 研究并解决的问题
-研究问题：我们从理论构建和理论检验两个维度介绍一个反映实证文献理论贡献的分类法。
-现实痛点/理论缺口：尽管有多种因素可以解释这一趋势，但一个可能的原因是实证文章缺乏充分描述一个理论(大麦, 2006)要素所需的空间。考虑到这一局限性，一篇实证文章究竟意味着什么，才能做出理论上的贡献。
-作者要“解决”的具体点：我们的研究目的有三。首先，我们创建了一个</t>
-        </is>
-      </c>
-      <c r="AA2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>skipped_existing_or_no_fields</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>generated</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>https://app.notion.com/p/Trends-in-Theory-Building-and-Theory-Testing-A-Five-Decade-Study-of-the-i-Academy-of-Management-Jo-395e8c8a654d815583dedaab8009b7b9</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>395e8c8a-654d-8155-83de-daab8009b7b9</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:23:33</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Methodological fit in management field research</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>管理领域研究中的方法论契合度</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Amy C. Edmondson; Stacy E. Mcmanus</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2007</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Academy of Management Review</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>10.5465/amr.2007.26586086</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>to-notion</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>已翻译</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>部分已翻译</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>已从 Zotero 导入</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>已同步</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="n">
-        <v>69</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>0. 文献名称
-Methodological fit in management field research
-1. 研究问题（Research Question）
-核心研究问题：方法匹配作为组织高质量实地研究的隐性价值属性，在管理学文献中很少受到关注。引入了一个权变框架，将先前的工作与研究项目的设计联系起来，特别关注在一篇研究论文中何时混合定性和定量数据的问题
-研究动机/现实背景：
-为了推进管理理论的发展，越来越多的学者从事实地研究，研究现实的人、现实的问题、现实的组织。虽然实地研究的潜在相关性是令人鼓舞的，但研究旅程可能是混乱和低效的，充满了逻辑障碍和意想不到的事件。研究人员管理与网站的复</t>
-        </is>
-      </c>
-      <c r="AA3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>skipped_existing_or_no_fields</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>generated</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>https://app.notion.com/p/Methodological-fit-in-management-field-research-395e8c8a654d81b69d3cce24cb21dc3a</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>395e8c8a-654d-81b6-9d3c-ce24cb21dc3a</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-07-07T09:23:33</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Building Theories from Case Study Research</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>从案例研究中构建理论</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Kathleen M Eisenhardt</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>to-notion</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>已翻译</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>部分已翻译</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>已从 Zotero 导入</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>已同步</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="n">
-        <v>132</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>0. 文献名称
-Building Theories from Case  Study Research
-1. 研究并解决的问题
-研究问题：本文描述了运用案例研究进行理论归纳的过程- -从明确研究问题到得出研究结论。该过程的一些特征，如问题界定、构念验证等，与假设检验研究有相似之处。另外一些，如案例内分析和复制逻辑，是归纳的、面向案例的过程所特有的。总的来说，这里描述的过程是高度迭代的，并且与数据紧密相连。这种研究方法在新的主题领域尤其适用。由此产生的理论往往是新颖的、可检验的和经验有效的。最后，卢德分子的洞见、(例如,简约性、逻辑连贯性)的良好理论的检验以及证据中的令人信服的基础是评价这类研究</t>
-        </is>
-      </c>
-      <c r="AA4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>skipped_existing_or_no_fields</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>generated</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>https://app.notion.com/p/Building-Theories-from-Case-Study-Research-395e8c8a654d814f96e6f7022871fd51</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>395e8c8a-654d-814f-96e6-f7022871fd51</t>
         </is>
       </c>
     </row>

</xml_diff>